<commit_message>
feat: add dedicated rule for keeping dishes out of the sink
</commit_message>
<xml_diff>
--- a/rozpis_sluzeb_byt.xlsx
+++ b/rozpis_sluzeb_byt.xlsx
@@ -5940,7 +5940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6457,7 +6457,7 @@
       </c>
       <c r="C49" s="69" t="inlineStr">
         <is>
-          <t>Služba neuklízí cizí nepořádek! Každý po sobě ihned utře linku, když něco rozlije, a umyje své věci.</t>
+          <t>Služba neuklízí cizí nepořádek! Každý po sobě ihned utře linku, když něco rozlije, a udržuje pořádek.</t>
         </is>
       </c>
       <c r="D49" s="70" t="n"/>
@@ -6472,20 +6472,40 @@
       </c>
       <c r="B50" s="68" t="inlineStr">
         <is>
-          <t>Spotřební materiál a chemie:</t>
+          <t>Žádné nádobí ve dřezu:</t>
         </is>
       </c>
       <c r="C50" s="69" t="inlineStr">
         <is>
-          <t>Když dochází jar, tablety do myčky, WC gel, toaletní papír nebo pytle do koše, tak to koupíš a hodíš do SettleUp.</t>
+          <t>Ve dřezu nesmí zůstávat nádobí – plný dřez se nedá používat. Při plné myčce odložit vedle na linku a pak do myčky, nebo hned umýt.</t>
         </is>
       </c>
       <c r="D50" s="70" t="n"/>
       <c r="E50" s="70" t="n"/>
       <c r="F50" s="70" t="n"/>
     </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="67" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="B51" s="68" t="inlineStr">
+        <is>
+          <t>Spotřební materiál a chemie:</t>
+        </is>
+      </c>
+      <c r="C51" s="69" t="inlineStr">
+        <is>
+          <t>Když dochází jar, tablety do myčky, WC gel, toaletní papír nebo pytle do koše, tak to koupíš a hodíš do SettleUp.</t>
+        </is>
+      </c>
+      <c r="D51" s="70" t="n"/>
+      <c r="E51" s="70" t="n"/>
+      <c r="F51" s="70" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="38">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="C48:F48"/>
     <mergeCell ref="A46:F46"/>
@@ -6519,6 +6539,7 @@
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B36:F36"/>
+    <mergeCell ref="C51:F51"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="A25:F25"/>

</xml_diff>

<commit_message>
feat: use ISO week numbers, auto-hide past weeks, refine chore details and rules
</commit_message>
<xml_diff>
--- a/rozpis_sluzeb_byt.xlsx
+++ b/rozpis_sluzeb_byt.xlsx
@@ -1123,10 +1123,9 @@
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Týden 1</t>
-        </is>
+      <c r="A7" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B7)</f>
+        <v/>
       </c>
       <c r="B7" s="12">
         <f>$B$4 + (0*7)</f>
@@ -1158,10 +1157,9 @@
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>Týden 2</t>
-        </is>
+      <c r="A8" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B8)</f>
+        <v/>
       </c>
       <c r="B8" s="15">
         <f>$B$4 + (1*7)</f>
@@ -1193,10 +1191,9 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Týden 3</t>
-        </is>
+      <c r="A9" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B9)</f>
+        <v/>
       </c>
       <c r="B9" s="12">
         <f>$B$4 + (2*7)</f>
@@ -1228,10 +1225,9 @@
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>Týden 4</t>
-        </is>
+      <c r="A10" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B10)</f>
+        <v/>
       </c>
       <c r="B10" s="15">
         <f>$B$4 + (3*7)</f>
@@ -1263,10 +1259,9 @@
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Týden 5</t>
-        </is>
+      <c r="A11" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B11)</f>
+        <v/>
       </c>
       <c r="B11" s="12">
         <f>$B$4 + (4*7)</f>
@@ -1298,10 +1293,9 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Týden 6</t>
-        </is>
+      <c r="A12" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B12)</f>
+        <v/>
       </c>
       <c r="B12" s="15">
         <f>$B$4 + (5*7)</f>
@@ -1333,10 +1327,9 @@
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Týden 7</t>
-        </is>
+      <c r="A13" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B13)</f>
+        <v/>
       </c>
       <c r="B13" s="12">
         <f>$B$4 + (6*7)</f>
@@ -1368,10 +1361,9 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Týden 8</t>
-        </is>
+      <c r="A14" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B14)</f>
+        <v/>
       </c>
       <c r="B14" s="15">
         <f>$B$4 + (7*7)</f>
@@ -1403,10 +1395,9 @@
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>Týden 9</t>
-        </is>
+      <c r="A15" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B15)</f>
+        <v/>
       </c>
       <c r="B15" s="12">
         <f>$B$4 + (8*7)</f>
@@ -1438,10 +1429,9 @@
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Týden 10</t>
-        </is>
+      <c r="A16" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B16)</f>
+        <v/>
       </c>
       <c r="B16" s="15">
         <f>$B$4 + (9*7)</f>
@@ -1473,10 +1463,9 @@
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>Týden 11</t>
-        </is>
+      <c r="A17" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B17)</f>
+        <v/>
       </c>
       <c r="B17" s="12">
         <f>$B$4 + (10*7)</f>
@@ -1508,10 +1497,9 @@
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Týden 12</t>
-        </is>
+      <c r="A18" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B18)</f>
+        <v/>
       </c>
       <c r="B18" s="15">
         <f>$B$4 + (11*7)</f>
@@ -1543,10 +1531,9 @@
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>Týden 13</t>
-        </is>
+      <c r="A19" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B19)</f>
+        <v/>
       </c>
       <c r="B19" s="12">
         <f>$B$4 + (12*7)</f>
@@ -1578,10 +1565,9 @@
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>Týden 14</t>
-        </is>
+      <c r="A20" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B20)</f>
+        <v/>
       </c>
       <c r="B20" s="15">
         <f>$B$4 + (13*7)</f>
@@ -1613,10 +1599,9 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>Týden 15</t>
-        </is>
+      <c r="A21" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B21)</f>
+        <v/>
       </c>
       <c r="B21" s="12">
         <f>$B$4 + (14*7)</f>
@@ -1648,10 +1633,9 @@
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>Týden 16</t>
-        </is>
+      <c r="A22" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B22)</f>
+        <v/>
       </c>
       <c r="B22" s="15">
         <f>$B$4 + (15*7)</f>
@@ -1683,10 +1667,9 @@
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>Týden 17</t>
-        </is>
+      <c r="A23" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B23)</f>
+        <v/>
       </c>
       <c r="B23" s="12">
         <f>$B$4 + (16*7)</f>
@@ -1718,10 +1701,9 @@
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>Týden 18</t>
-        </is>
+      <c r="A24" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B24)</f>
+        <v/>
       </c>
       <c r="B24" s="15">
         <f>$B$4 + (17*7)</f>
@@ -1753,10 +1735,9 @@
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>Týden 19</t>
-        </is>
+      <c r="A25" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B25)</f>
+        <v/>
       </c>
       <c r="B25" s="12">
         <f>$B$4 + (18*7)</f>
@@ -1788,10 +1769,9 @@
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="14" t="inlineStr">
-        <is>
-          <t>Týden 20</t>
-        </is>
+      <c r="A26" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B26)</f>
+        <v/>
       </c>
       <c r="B26" s="15">
         <f>$B$4 + (19*7)</f>
@@ -1823,10 +1803,9 @@
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>Týden 21</t>
-        </is>
+      <c r="A27" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B27)</f>
+        <v/>
       </c>
       <c r="B27" s="12">
         <f>$B$4 + (20*7)</f>
@@ -1858,10 +1837,9 @@
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
-        <is>
-          <t>Týden 22</t>
-        </is>
+      <c r="A28" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B28)</f>
+        <v/>
       </c>
       <c r="B28" s="15">
         <f>$B$4 + (21*7)</f>
@@ -1893,10 +1871,9 @@
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>Týden 23</t>
-        </is>
+      <c r="A29" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B29)</f>
+        <v/>
       </c>
       <c r="B29" s="12">
         <f>$B$4 + (22*7)</f>
@@ -1928,10 +1905,9 @@
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
-        <is>
-          <t>Týden 24</t>
-        </is>
+      <c r="A30" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B30)</f>
+        <v/>
       </c>
       <c r="B30" s="15">
         <f>$B$4 + (23*7)</f>
@@ -1963,10 +1939,9 @@
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>Týden 25</t>
-        </is>
+      <c r="A31" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B31)</f>
+        <v/>
       </c>
       <c r="B31" s="12">
         <f>$B$4 + (24*7)</f>
@@ -1998,10 +1973,9 @@
       </c>
     </row>
     <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="14" t="inlineStr">
-        <is>
-          <t>Týden 26</t>
-        </is>
+      <c r="A32" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B32)</f>
+        <v/>
       </c>
       <c r="B32" s="15">
         <f>$B$4 + (25*7)</f>
@@ -2033,10 +2007,9 @@
       </c>
     </row>
     <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>Týden 27</t>
-        </is>
+      <c r="A33" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B33)</f>
+        <v/>
       </c>
       <c r="B33" s="12">
         <f>$B$4 + (26*7)</f>
@@ -2068,10 +2041,9 @@
       </c>
     </row>
     <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="14" t="inlineStr">
-        <is>
-          <t>Týden 28</t>
-        </is>
+      <c r="A34" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B34)</f>
+        <v/>
       </c>
       <c r="B34" s="15">
         <f>$B$4 + (27*7)</f>
@@ -2103,10 +2075,9 @@
       </c>
     </row>
     <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>Týden 29</t>
-        </is>
+      <c r="A35" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B35)</f>
+        <v/>
       </c>
       <c r="B35" s="12">
         <f>$B$4 + (28*7)</f>
@@ -2138,10 +2109,9 @@
       </c>
     </row>
     <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>Týden 30</t>
-        </is>
+      <c r="A36" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B36)</f>
+        <v/>
       </c>
       <c r="B36" s="15">
         <f>$B$4 + (29*7)</f>
@@ -2173,10 +2143,9 @@
       </c>
     </row>
     <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t>Týden 31</t>
-        </is>
+      <c r="A37" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B37)</f>
+        <v/>
       </c>
       <c r="B37" s="12">
         <f>$B$4 + (30*7)</f>
@@ -2208,10 +2177,9 @@
       </c>
     </row>
     <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
-        <is>
-          <t>Týden 32</t>
-        </is>
+      <c r="A38" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B38)</f>
+        <v/>
       </c>
       <c r="B38" s="15">
         <f>$B$4 + (31*7)</f>
@@ -2243,10 +2211,9 @@
       </c>
     </row>
     <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>Týden 33</t>
-        </is>
+      <c r="A39" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B39)</f>
+        <v/>
       </c>
       <c r="B39" s="12">
         <f>$B$4 + (32*7)</f>
@@ -2278,10 +2245,9 @@
       </c>
     </row>
     <row r="40" ht="24" customHeight="1">
-      <c r="A40" s="14" t="inlineStr">
-        <is>
-          <t>Týden 34</t>
-        </is>
+      <c r="A40" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B40)</f>
+        <v/>
       </c>
       <c r="B40" s="15">
         <f>$B$4 + (33*7)</f>
@@ -2313,10 +2279,9 @@
       </c>
     </row>
     <row r="41" ht="24" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>Týden 35</t>
-        </is>
+      <c r="A41" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B41)</f>
+        <v/>
       </c>
       <c r="B41" s="12">
         <f>$B$4 + (34*7)</f>
@@ -2348,10 +2313,9 @@
       </c>
     </row>
     <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="14" t="inlineStr">
-        <is>
-          <t>Týden 36</t>
-        </is>
+      <c r="A42" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B42)</f>
+        <v/>
       </c>
       <c r="B42" s="15">
         <f>$B$4 + (35*7)</f>
@@ -2383,10 +2347,9 @@
       </c>
     </row>
     <row r="43" ht="24" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>Týden 37</t>
-        </is>
+      <c r="A43" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B43)</f>
+        <v/>
       </c>
       <c r="B43" s="12">
         <f>$B$4 + (36*7)</f>
@@ -2418,10 +2381,9 @@
       </c>
     </row>
     <row r="44" ht="24" customHeight="1">
-      <c r="A44" s="14" t="inlineStr">
-        <is>
-          <t>Týden 38</t>
-        </is>
+      <c r="A44" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B44)</f>
+        <v/>
       </c>
       <c r="B44" s="15">
         <f>$B$4 + (37*7)</f>
@@ -2453,10 +2415,9 @@
       </c>
     </row>
     <row r="45" ht="24" customHeight="1">
-      <c r="A45" s="11" t="inlineStr">
-        <is>
-          <t>Týden 39</t>
-        </is>
+      <c r="A45" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B45)</f>
+        <v/>
       </c>
       <c r="B45" s="12">
         <f>$B$4 + (38*7)</f>
@@ -2488,10 +2449,9 @@
       </c>
     </row>
     <row r="46" ht="24" customHeight="1">
-      <c r="A46" s="14" t="inlineStr">
-        <is>
-          <t>Týden 40</t>
-        </is>
+      <c r="A46" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B46)</f>
+        <v/>
       </c>
       <c r="B46" s="15">
         <f>$B$4 + (39*7)</f>
@@ -2523,10 +2483,9 @@
       </c>
     </row>
     <row r="47" ht="24" customHeight="1">
-      <c r="A47" s="11" t="inlineStr">
-        <is>
-          <t>Týden 41</t>
-        </is>
+      <c r="A47" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B47)</f>
+        <v/>
       </c>
       <c r="B47" s="12">
         <f>$B$4 + (40*7)</f>
@@ -2558,10 +2517,9 @@
       </c>
     </row>
     <row r="48" ht="24" customHeight="1">
-      <c r="A48" s="14" t="inlineStr">
-        <is>
-          <t>Týden 42</t>
-        </is>
+      <c r="A48" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B48)</f>
+        <v/>
       </c>
       <c r="B48" s="15">
         <f>$B$4 + (41*7)</f>
@@ -2593,10 +2551,9 @@
       </c>
     </row>
     <row r="49" ht="24" customHeight="1">
-      <c r="A49" s="11" t="inlineStr">
-        <is>
-          <t>Týden 43</t>
-        </is>
+      <c r="A49" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B49)</f>
+        <v/>
       </c>
       <c r="B49" s="12">
         <f>$B$4 + (42*7)</f>
@@ -2628,10 +2585,9 @@
       </c>
     </row>
     <row r="50" ht="24" customHeight="1">
-      <c r="A50" s="14" t="inlineStr">
-        <is>
-          <t>Týden 44</t>
-        </is>
+      <c r="A50" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B50)</f>
+        <v/>
       </c>
       <c r="B50" s="15">
         <f>$B$4 + (43*7)</f>
@@ -2663,10 +2619,9 @@
       </c>
     </row>
     <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="11" t="inlineStr">
-        <is>
-          <t>Týden 45</t>
-        </is>
+      <c r="A51" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B51)</f>
+        <v/>
       </c>
       <c r="B51" s="12">
         <f>$B$4 + (44*7)</f>
@@ -2698,10 +2653,9 @@
       </c>
     </row>
     <row r="52" ht="24" customHeight="1">
-      <c r="A52" s="14" t="inlineStr">
-        <is>
-          <t>Týden 46</t>
-        </is>
+      <c r="A52" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B52)</f>
+        <v/>
       </c>
       <c r="B52" s="15">
         <f>$B$4 + (45*7)</f>
@@ -2733,10 +2687,9 @@
       </c>
     </row>
     <row r="53" ht="24" customHeight="1">
-      <c r="A53" s="11" t="inlineStr">
-        <is>
-          <t>Týden 47</t>
-        </is>
+      <c r="A53" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B53)</f>
+        <v/>
       </c>
       <c r="B53" s="12">
         <f>$B$4 + (46*7)</f>
@@ -2768,10 +2721,9 @@
       </c>
     </row>
     <row r="54" ht="24" customHeight="1">
-      <c r="A54" s="14" t="inlineStr">
-        <is>
-          <t>Týden 48</t>
-        </is>
+      <c r="A54" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B54)</f>
+        <v/>
       </c>
       <c r="B54" s="15">
         <f>$B$4 + (47*7)</f>
@@ -2803,10 +2755,9 @@
       </c>
     </row>
     <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>Týden 49</t>
-        </is>
+      <c r="A55" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B55)</f>
+        <v/>
       </c>
       <c r="B55" s="12">
         <f>$B$4 + (48*7)</f>
@@ -2838,10 +2789,9 @@
       </c>
     </row>
     <row r="56" ht="24" customHeight="1">
-      <c r="A56" s="14" t="inlineStr">
-        <is>
-          <t>Týden 50</t>
-        </is>
+      <c r="A56" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B56)</f>
+        <v/>
       </c>
       <c r="B56" s="15">
         <f>$B$4 + (49*7)</f>
@@ -2873,10 +2823,9 @@
       </c>
     </row>
     <row r="57" ht="24" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
-        <is>
-          <t>Týden 51</t>
-        </is>
+      <c r="A57" s="11">
+        <f>"Týden " &amp; ISOWEEKNUM(B57)</f>
+        <v/>
       </c>
       <c r="B57" s="12">
         <f>$B$4 + (50*7)</f>
@@ -2908,10 +2857,9 @@
       </c>
     </row>
     <row r="58" ht="24" customHeight="1">
-      <c r="A58" s="14" t="inlineStr">
-        <is>
-          <t>Týden 52</t>
-        </is>
+      <c r="A58" s="14">
+        <f>"Týden " &amp; ISOWEEKNUM(B58)</f>
+        <v/>
       </c>
       <c r="B58" s="15">
         <f>$B$4 + (51*7)</f>
@@ -3063,10 +3011,9 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Týden 1</t>
-        </is>
+      <c r="A6" s="11">
+        <f>'Rozpis podle pokojů'!A7</f>
+        <v/>
       </c>
       <c r="B6" s="22">
         <f>'Rozpis podle pokojů'!B7</f>
@@ -3118,10 +3065,9 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Týden 2</t>
-        </is>
+      <c r="A7" s="14">
+        <f>'Rozpis podle pokojů'!A8</f>
+        <v/>
       </c>
       <c r="B7" s="27">
         <f>'Rozpis podle pokojů'!B8</f>
@@ -3173,10 +3119,9 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Týden 3</t>
-        </is>
+      <c r="A8" s="11">
+        <f>'Rozpis podle pokojů'!A9</f>
+        <v/>
       </c>
       <c r="B8" s="22">
         <f>'Rozpis podle pokojů'!B9</f>
@@ -3228,10 +3173,9 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>Týden 4</t>
-        </is>
+      <c r="A9" s="14">
+        <f>'Rozpis podle pokojů'!A10</f>
+        <v/>
       </c>
       <c r="B9" s="27">
         <f>'Rozpis podle pokojů'!B10</f>
@@ -3283,10 +3227,9 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>Týden 5</t>
-        </is>
+      <c r="A10" s="11">
+        <f>'Rozpis podle pokojů'!A11</f>
+        <v/>
       </c>
       <c r="B10" s="22">
         <f>'Rozpis podle pokojů'!B11</f>
@@ -3338,10 +3281,9 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Týden 6</t>
-        </is>
+      <c r="A11" s="14">
+        <f>'Rozpis podle pokojů'!A12</f>
+        <v/>
       </c>
       <c r="B11" s="27">
         <f>'Rozpis podle pokojů'!B12</f>
@@ -3393,10 +3335,9 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Týden 7</t>
-        </is>
+      <c r="A12" s="11">
+        <f>'Rozpis podle pokojů'!A13</f>
+        <v/>
       </c>
       <c r="B12" s="22">
         <f>'Rozpis podle pokojů'!B13</f>
@@ -3448,10 +3389,9 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>Týden 8</t>
-        </is>
+      <c r="A13" s="14">
+        <f>'Rozpis podle pokojů'!A14</f>
+        <v/>
       </c>
       <c r="B13" s="27">
         <f>'Rozpis podle pokojů'!B14</f>
@@ -3503,10 +3443,9 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>Týden 9</t>
-        </is>
+      <c r="A14" s="11">
+        <f>'Rozpis podle pokojů'!A15</f>
+        <v/>
       </c>
       <c r="B14" s="22">
         <f>'Rozpis podle pokojů'!B15</f>
@@ -3558,10 +3497,9 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>Týden 10</t>
-        </is>
+      <c r="A15" s="14">
+        <f>'Rozpis podle pokojů'!A16</f>
+        <v/>
       </c>
       <c r="B15" s="27">
         <f>'Rozpis podle pokojů'!B16</f>
@@ -3613,10 +3551,9 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>Týden 11</t>
-        </is>
+      <c r="A16" s="11">
+        <f>'Rozpis podle pokojů'!A17</f>
+        <v/>
       </c>
       <c r="B16" s="22">
         <f>'Rozpis podle pokojů'!B17</f>
@@ -3668,10 +3605,9 @@
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>Týden 12</t>
-        </is>
+      <c r="A17" s="14">
+        <f>'Rozpis podle pokojů'!A18</f>
+        <v/>
       </c>
       <c r="B17" s="27">
         <f>'Rozpis podle pokojů'!B18</f>
@@ -3723,10 +3659,9 @@
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>Týden 13</t>
-        </is>
+      <c r="A18" s="11">
+        <f>'Rozpis podle pokojů'!A19</f>
+        <v/>
       </c>
       <c r="B18" s="22">
         <f>'Rozpis podle pokojů'!B19</f>
@@ -3778,10 +3713,9 @@
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>Týden 14</t>
-        </is>
+      <c r="A19" s="14">
+        <f>'Rozpis podle pokojů'!A20</f>
+        <v/>
       </c>
       <c r="B19" s="27">
         <f>'Rozpis podle pokojů'!B20</f>
@@ -3833,10 +3767,9 @@
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>Týden 15</t>
-        </is>
+      <c r="A20" s="11">
+        <f>'Rozpis podle pokojů'!A21</f>
+        <v/>
       </c>
       <c r="B20" s="22">
         <f>'Rozpis podle pokojů'!B21</f>
@@ -3888,10 +3821,9 @@
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>Týden 16</t>
-        </is>
+      <c r="A21" s="14">
+        <f>'Rozpis podle pokojů'!A22</f>
+        <v/>
       </c>
       <c r="B21" s="27">
         <f>'Rozpis podle pokojů'!B22</f>
@@ -3943,10 +3875,9 @@
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Týden 17</t>
-        </is>
+      <c r="A22" s="11">
+        <f>'Rozpis podle pokojů'!A23</f>
+        <v/>
       </c>
       <c r="B22" s="22">
         <f>'Rozpis podle pokojů'!B23</f>
@@ -3998,10 +3929,9 @@
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t>Týden 18</t>
-        </is>
+      <c r="A23" s="14">
+        <f>'Rozpis podle pokojů'!A24</f>
+        <v/>
       </c>
       <c r="B23" s="27">
         <f>'Rozpis podle pokojů'!B24</f>
@@ -4053,10 +3983,9 @@
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>Týden 19</t>
-        </is>
+      <c r="A24" s="11">
+        <f>'Rozpis podle pokojů'!A25</f>
+        <v/>
       </c>
       <c r="B24" s="22">
         <f>'Rozpis podle pokojů'!B25</f>
@@ -4108,10 +4037,9 @@
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="14" t="inlineStr">
-        <is>
-          <t>Týden 20</t>
-        </is>
+      <c r="A25" s="14">
+        <f>'Rozpis podle pokojů'!A26</f>
+        <v/>
       </c>
       <c r="B25" s="27">
         <f>'Rozpis podle pokojů'!B26</f>
@@ -4163,10 +4091,9 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>Týden 21</t>
-        </is>
+      <c r="A26" s="11">
+        <f>'Rozpis podle pokojů'!A27</f>
+        <v/>
       </c>
       <c r="B26" s="22">
         <f>'Rozpis podle pokojů'!B27</f>
@@ -4218,10 +4145,9 @@
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>Týden 22</t>
-        </is>
+      <c r="A27" s="14">
+        <f>'Rozpis podle pokojů'!A28</f>
+        <v/>
       </c>
       <c r="B27" s="27">
         <f>'Rozpis podle pokojů'!B28</f>
@@ -4273,10 +4199,9 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>Týden 23</t>
-        </is>
+      <c r="A28" s="11">
+        <f>'Rozpis podle pokojů'!A29</f>
+        <v/>
       </c>
       <c r="B28" s="22">
         <f>'Rozpis podle pokojů'!B29</f>
@@ -4328,10 +4253,9 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
-        <is>
-          <t>Týden 24</t>
-        </is>
+      <c r="A29" s="14">
+        <f>'Rozpis podle pokojů'!A30</f>
+        <v/>
       </c>
       <c r="B29" s="27">
         <f>'Rozpis podle pokojů'!B30</f>
@@ -4383,10 +4307,9 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>Týden 25</t>
-        </is>
+      <c r="A30" s="11">
+        <f>'Rozpis podle pokojů'!A31</f>
+        <v/>
       </c>
       <c r="B30" s="22">
         <f>'Rozpis podle pokojů'!B31</f>
@@ -4438,10 +4361,9 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
-        <is>
-          <t>Týden 26</t>
-        </is>
+      <c r="A31" s="14">
+        <f>'Rozpis podle pokojů'!A32</f>
+        <v/>
       </c>
       <c r="B31" s="27">
         <f>'Rozpis podle pokojů'!B32</f>
@@ -4493,10 +4415,9 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>Týden 27</t>
-        </is>
+      <c r="A32" s="11">
+        <f>'Rozpis podle pokojů'!A33</f>
+        <v/>
       </c>
       <c r="B32" s="22">
         <f>'Rozpis podle pokojů'!B33</f>
@@ -4548,10 +4469,9 @@
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>Týden 28</t>
-        </is>
+      <c r="A33" s="14">
+        <f>'Rozpis podle pokojů'!A34</f>
+        <v/>
       </c>
       <c r="B33" s="27">
         <f>'Rozpis podle pokojů'!B34</f>
@@ -4603,10 +4523,9 @@
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="11" t="inlineStr">
-        <is>
-          <t>Týden 29</t>
-        </is>
+      <c r="A34" s="11">
+        <f>'Rozpis podle pokojů'!A35</f>
+        <v/>
       </c>
       <c r="B34" s="22">
         <f>'Rozpis podle pokojů'!B35</f>
@@ -4658,10 +4577,9 @@
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="14" t="inlineStr">
-        <is>
-          <t>Týden 30</t>
-        </is>
+      <c r="A35" s="14">
+        <f>'Rozpis podle pokojů'!A36</f>
+        <v/>
       </c>
       <c r="B35" s="27">
         <f>'Rozpis podle pokojů'!B36</f>
@@ -4713,10 +4631,9 @@
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
-        <is>
-          <t>Týden 31</t>
-        </is>
+      <c r="A36" s="11">
+        <f>'Rozpis podle pokojů'!A37</f>
+        <v/>
       </c>
       <c r="B36" s="22">
         <f>'Rozpis podle pokojů'!B37</f>
@@ -4768,10 +4685,9 @@
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="14" t="inlineStr">
-        <is>
-          <t>Týden 32</t>
-        </is>
+      <c r="A37" s="14">
+        <f>'Rozpis podle pokojů'!A38</f>
+        <v/>
       </c>
       <c r="B37" s="27">
         <f>'Rozpis podle pokojů'!B38</f>
@@ -4823,10 +4739,9 @@
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>Týden 33</t>
-        </is>
+      <c r="A38" s="11">
+        <f>'Rozpis podle pokojů'!A39</f>
+        <v/>
       </c>
       <c r="B38" s="22">
         <f>'Rozpis podle pokojů'!B39</f>
@@ -4878,10 +4793,9 @@
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>Týden 34</t>
-        </is>
+      <c r="A39" s="14">
+        <f>'Rozpis podle pokojů'!A40</f>
+        <v/>
       </c>
       <c r="B39" s="27">
         <f>'Rozpis podle pokojů'!B40</f>
@@ -4933,10 +4847,9 @@
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>Týden 35</t>
-        </is>
+      <c r="A40" s="11">
+        <f>'Rozpis podle pokojů'!A41</f>
+        <v/>
       </c>
       <c r="B40" s="22">
         <f>'Rozpis podle pokojů'!B41</f>
@@ -4988,10 +4901,9 @@
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="14" t="inlineStr">
-        <is>
-          <t>Týden 36</t>
-        </is>
+      <c r="A41" s="14">
+        <f>'Rozpis podle pokojů'!A42</f>
+        <v/>
       </c>
       <c r="B41" s="27">
         <f>'Rozpis podle pokojů'!B42</f>
@@ -5043,10 +4955,9 @@
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
-        <is>
-          <t>Týden 37</t>
-        </is>
+      <c r="A42" s="11">
+        <f>'Rozpis podle pokojů'!A43</f>
+        <v/>
       </c>
       <c r="B42" s="22">
         <f>'Rozpis podle pokojů'!B43</f>
@@ -5098,10 +5009,9 @@
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="14" t="inlineStr">
-        <is>
-          <t>Týden 38</t>
-        </is>
+      <c r="A43" s="14">
+        <f>'Rozpis podle pokojů'!A44</f>
+        <v/>
       </c>
       <c r="B43" s="27">
         <f>'Rozpis podle pokojů'!B44</f>
@@ -5153,10 +5063,9 @@
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
-        <is>
-          <t>Týden 39</t>
-        </is>
+      <c r="A44" s="11">
+        <f>'Rozpis podle pokojů'!A45</f>
+        <v/>
       </c>
       <c r="B44" s="22">
         <f>'Rozpis podle pokojů'!B45</f>
@@ -5208,10 +5117,9 @@
       </c>
     </row>
     <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="14" t="inlineStr">
-        <is>
-          <t>Týden 40</t>
-        </is>
+      <c r="A45" s="14">
+        <f>'Rozpis podle pokojů'!A46</f>
+        <v/>
       </c>
       <c r="B45" s="27">
         <f>'Rozpis podle pokojů'!B46</f>
@@ -5263,10 +5171,9 @@
       </c>
     </row>
     <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
-        <is>
-          <t>Týden 41</t>
-        </is>
+      <c r="A46" s="11">
+        <f>'Rozpis podle pokojů'!A47</f>
+        <v/>
       </c>
       <c r="B46" s="22">
         <f>'Rozpis podle pokojů'!B47</f>
@@ -5318,10 +5225,9 @@
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="14" t="inlineStr">
-        <is>
-          <t>Týden 42</t>
-        </is>
+      <c r="A47" s="14">
+        <f>'Rozpis podle pokojů'!A48</f>
+        <v/>
       </c>
       <c r="B47" s="27">
         <f>'Rozpis podle pokojů'!B48</f>
@@ -5373,10 +5279,9 @@
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="11" t="inlineStr">
-        <is>
-          <t>Týden 43</t>
-        </is>
+      <c r="A48" s="11">
+        <f>'Rozpis podle pokojů'!A49</f>
+        <v/>
       </c>
       <c r="B48" s="22">
         <f>'Rozpis podle pokojů'!B49</f>
@@ -5428,10 +5333,9 @@
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="14" t="inlineStr">
-        <is>
-          <t>Týden 44</t>
-        </is>
+      <c r="A49" s="14">
+        <f>'Rozpis podle pokojů'!A50</f>
+        <v/>
       </c>
       <c r="B49" s="27">
         <f>'Rozpis podle pokojů'!B50</f>
@@ -5483,10 +5387,9 @@
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="11" t="inlineStr">
-        <is>
-          <t>Týden 45</t>
-        </is>
+      <c r="A50" s="11">
+        <f>'Rozpis podle pokojů'!A51</f>
+        <v/>
       </c>
       <c r="B50" s="22">
         <f>'Rozpis podle pokojů'!B51</f>
@@ -5538,10 +5441,9 @@
       </c>
     </row>
     <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="14" t="inlineStr">
-        <is>
-          <t>Týden 46</t>
-        </is>
+      <c r="A51" s="14">
+        <f>'Rozpis podle pokojů'!A52</f>
+        <v/>
       </c>
       <c r="B51" s="27">
         <f>'Rozpis podle pokojů'!B52</f>
@@ -5593,10 +5495,9 @@
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="11" t="inlineStr">
-        <is>
-          <t>Týden 47</t>
-        </is>
+      <c r="A52" s="11">
+        <f>'Rozpis podle pokojů'!A53</f>
+        <v/>
       </c>
       <c r="B52" s="22">
         <f>'Rozpis podle pokojů'!B53</f>
@@ -5648,10 +5549,9 @@
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="14" t="inlineStr">
-        <is>
-          <t>Týden 48</t>
-        </is>
+      <c r="A53" s="14">
+        <f>'Rozpis podle pokojů'!A54</f>
+        <v/>
       </c>
       <c r="B53" s="27">
         <f>'Rozpis podle pokojů'!B54</f>
@@ -5703,10 +5603,9 @@
       </c>
     </row>
     <row r="54" ht="22" customHeight="1">
-      <c r="A54" s="11" t="inlineStr">
-        <is>
-          <t>Týden 49</t>
-        </is>
+      <c r="A54" s="11">
+        <f>'Rozpis podle pokojů'!A55</f>
+        <v/>
       </c>
       <c r="B54" s="22">
         <f>'Rozpis podle pokojů'!B55</f>
@@ -5758,10 +5657,9 @@
       </c>
     </row>
     <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="14" t="inlineStr">
-        <is>
-          <t>Týden 50</t>
-        </is>
+      <c r="A55" s="14">
+        <f>'Rozpis podle pokojů'!A56</f>
+        <v/>
       </c>
       <c r="B55" s="27">
         <f>'Rozpis podle pokojů'!B56</f>
@@ -5813,10 +5711,9 @@
       </c>
     </row>
     <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="11" t="inlineStr">
-        <is>
-          <t>Týden 51</t>
-        </is>
+      <c r="A56" s="11">
+        <f>'Rozpis podle pokojů'!A57</f>
+        <v/>
       </c>
       <c r="B56" s="22">
         <f>'Rozpis podle pokojů'!B57</f>
@@ -5868,10 +5765,9 @@
       </c>
     </row>
     <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="14" t="inlineStr">
-        <is>
-          <t>Týden 52</t>
-        </is>
+      <c r="A57" s="14">
+        <f>'Rozpis podle pokojů'!A58</f>
+        <v/>
       </c>
       <c r="B57" s="27">
         <f>'Rozpis podle pokojů'!B58</f>
@@ -5940,7 +5836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6011,43 +5907,43 @@
       </c>
       <c r="B7" s="32" t="inlineStr">
         <is>
-          <t>Zkontrolovat, že na mezipatře / schodech nezůstaly žádné odpadky, letáky nebo kamínky.</t>
+          <t>Zkontrolovat, že na mezipatře / schodech nezůstaly žádné odpadky ani nepořádek.</t>
         </is>
       </c>
       <c r="F7" s="33" t="n"/>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+    <row r="8" ht="6" customHeight="1">
+      <c r="A8" s="34" t="n"/>
+      <c r="B8" s="35" t="n"/>
+      <c r="C8" s="35" t="n"/>
+      <c r="D8" s="35" t="n"/>
+      <c r="E8" s="35" t="n"/>
+      <c r="F8" s="36" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>🍳  KUCHYŇ   —   (Společná zóna vaření)</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="n"/>
+      <c r="C10" s="38" t="n"/>
+      <c r="D10" s="38" t="n"/>
+      <c r="E10" s="38" t="n"/>
+      <c r="F10" s="39" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B8" s="32" t="inlineStr">
-        <is>
-          <t>Doporučený čas splnění: pátek odpoledne nebo sobota dopoledne.</t>
-        </is>
-      </c>
-      <c r="F8" s="33" t="n"/>
-    </row>
-    <row r="9" ht="6" customHeight="1">
-      <c r="A9" s="34" t="n"/>
-      <c r="B9" s="35" t="n"/>
-      <c r="C9" s="35" t="n"/>
-      <c r="D9" s="35" t="n"/>
-      <c r="E9" s="35" t="n"/>
-      <c r="F9" s="36" t="n"/>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="37" t="inlineStr">
-        <is>
-          <t>🍳  KUCHYŇ   —   (Společná zóna vaření)</t>
-        </is>
-      </c>
-      <c r="B11" s="38" t="n"/>
-      <c r="C11" s="38" t="n"/>
-      <c r="D11" s="38" t="n"/>
-      <c r="E11" s="38" t="n"/>
-      <c r="F11" s="39" t="n"/>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>Starat se o kuchyňskou linku, dřez a varnou desku (otírat mastnotu a drobky).</t>
+        </is>
+      </c>
+      <c r="F11" s="40" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="31" t="inlineStr">
@@ -6057,7 +5953,7 @@
       </c>
       <c r="B12" s="32" t="inlineStr">
         <is>
-          <t>Starat se o kuchyňskou linku, dřez a varnou desku (otírat mastnotu a drobky).</t>
+          <t>Průběžně vyndávat umytou myčku a uklízet nádobí do skříněk.</t>
         </is>
       </c>
       <c r="F12" s="40" t="n"/>
@@ -6070,7 +5966,7 @@
       </c>
       <c r="B13" s="32" t="inlineStr">
         <is>
-          <t>Průběžně vyndávat umytou myčku a uklízet nádobí do skříněk.</t>
+          <t>Zapnout myčku, jakmile se naplní (nenechávat špinavé nádobí hromadit ve dřezu).</t>
         </is>
       </c>
       <c r="F13" s="40" t="n"/>
@@ -6083,43 +5979,43 @@
       </c>
       <c r="B14" s="32" t="inlineStr">
         <is>
-          <t>Zapnout myčku, jakmile se naplní (nenechávat špinavé nádobí hromadit ve dřezu).</t>
+          <t>Pravidelně zametat a vytírat podlahu v kuchyni (dle potřeby i v týdnu, min. 1× důkladně na závěr).</t>
         </is>
       </c>
       <c r="F14" s="40" t="n"/>
     </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="31" t="inlineStr">
+    <row r="15" ht="6" customHeight="1">
+      <c r="A15" s="41" t="n"/>
+      <c r="B15" s="42" t="n"/>
+      <c r="C15" s="42" t="n"/>
+      <c r="D15" s="42" t="n"/>
+      <c r="E15" s="42" t="n"/>
+      <c r="F15" s="43" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="44" t="inlineStr">
+        <is>
+          <t>🗑️  ODPADKY   —   (Čistý a voňavý byt)</t>
+        </is>
+      </c>
+      <c r="B17" s="45" t="n"/>
+      <c r="C17" s="45" t="n"/>
+      <c r="D17" s="45" t="n"/>
+      <c r="E17" s="45" t="n"/>
+      <c r="F17" s="46" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t>Pravidelně zametat a vytírat podlahu v kuchyni (dle potřeby i v týdnu, min. 1× důkladně na závěr).</t>
-        </is>
-      </c>
-      <c r="F15" s="40" t="n"/>
-    </row>
-    <row r="16" ht="6" customHeight="1">
-      <c r="A16" s="41" t="n"/>
-      <c r="B16" s="42" t="n"/>
-      <c r="C16" s="42" t="n"/>
-      <c r="D16" s="42" t="n"/>
-      <c r="E16" s="42" t="n"/>
-      <c r="F16" s="43" t="n"/>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="44" t="inlineStr">
-        <is>
-          <t>🗑️  ODPADKY   —   (Čistý a voňavý byt)</t>
-        </is>
-      </c>
-      <c r="B18" s="45" t="n"/>
-      <c r="C18" s="45" t="n"/>
-      <c r="D18" s="45" t="n"/>
-      <c r="E18" s="45" t="n"/>
-      <c r="F18" s="46" t="n"/>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>Pravidelně vynášet pytle se směsným odpadem, jakmile jsou plné (nečekat na přetečení).</t>
+        </is>
+      </c>
+      <c r="F18" s="47" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="31" t="inlineStr">
@@ -6129,7 +6025,7 @@
       </c>
       <c r="B19" s="32" t="inlineStr">
         <is>
-          <t>Pravidelně vynášet pytle se směsným odpadem, jakmile jsou plné (nečekat na přetečení).</t>
+          <t>Po vynesení koše VŽDY ihned nasadit nový čistý pytel!</t>
         </is>
       </c>
       <c r="F19" s="47" t="n"/>
@@ -6142,7 +6038,7 @@
       </c>
       <c r="B20" s="32" t="inlineStr">
         <is>
-          <t>Po vynesení koše VŽDY ihned nasadit nový čistý pytel!</t>
+          <t>Vynášet tříděný odpad (plast, papír, plechovky, sklo) do příslušných kontejnerů.</t>
         </is>
       </c>
       <c r="F20" s="47" t="n"/>
@@ -6155,7 +6051,7 @@
       </c>
       <c r="B21" s="32" t="inlineStr">
         <is>
-          <t>Vynášet tříděný odpad (plast, papír, plechovky, sklo) do příslušných kontejnerů.</t>
+          <t>Umýt odpadkový koš, pokud prosákl pytel nebo někdo něco hodil vedle.</t>
         </is>
       </c>
       <c r="F21" s="47" t="n"/>
@@ -6286,7 +6182,7 @@
       </c>
       <c r="B34" s="32" t="inlineStr">
         <is>
-          <t>Důkladně vymýt sprchový kout / vanu a odstranit vlasy ze sítka/odpadu.</t>
+          <t>Důkladně vymýt sprchový kout a vyčistit sítko od vlasů.</t>
         </is>
       </c>
       <c r="F34" s="33" t="n"/>
@@ -6412,12 +6308,12 @@
       </c>
       <c r="B47" s="68" t="inlineStr">
         <is>
-          <t>Předání služeb:</t>
+          <t>Průběžný pořádek:</t>
         </is>
       </c>
       <c r="C47" s="69" t="inlineStr">
         <is>
-          <t>Služba se oficiálně předává v NEDĚLI do 20:00 (do té doby je vše hotovo).</t>
+          <t>Služba neslouží jako osobní uklízeč! Každý po sobě ihned utře linku, když něco rozlije nebo rozsype, a udržuje společné prostory v čistotě.</t>
         </is>
       </c>
       <c r="D47" s="70" t="n"/>
@@ -6432,12 +6328,12 @@
       </c>
       <c r="B48" s="68" t="inlineStr">
         <is>
-          <t>Nepřítomnost:</t>
+          <t>Žádné nádobí ve dřezu:</t>
         </is>
       </c>
       <c r="C48" s="69" t="inlineStr">
         <is>
-          <t>Když někdo odjíždí na týden pryč, je jeho povinností si zajistit výměnu s jiným pokojem.</t>
+          <t>Ve dřezu nesmí zůstávat žádné nádobí – plný dřez se pak nedá vůbec používat. Při plné myčce odložit vedle na linku a po vyklizení dát do myčky, nebo hned umýt.</t>
         </is>
       </c>
       <c r="D48" s="70" t="n"/>
@@ -6452,12 +6348,12 @@
       </c>
       <c r="B49" s="68" t="inlineStr">
         <is>
-          <t>Průběžný pořádek:</t>
+          <t>Nepřítomnost a odjezdy:</t>
         </is>
       </c>
       <c r="C49" s="69" t="inlineStr">
         <is>
-          <t>Služba neuklízí cizí nepořádek! Každý po sobě ihned utře linku, když něco rozlije, a udržuje pořádek.</t>
+          <t>Když někdo odjíždí na týden pryč, je jeho povinností si zajistit výměnu s jiným pokojem.</t>
         </is>
       </c>
       <c r="D49" s="70" t="n"/>
@@ -6472,57 +6368,39 @@
       </c>
       <c r="B50" s="68" t="inlineStr">
         <is>
-          <t>Žádné nádobí ve dřezu:</t>
+          <t>Spotřební materiál a chemie:</t>
         </is>
       </c>
       <c r="C50" s="69" t="inlineStr">
         <is>
-          <t>Ve dřezu nesmí zůstávat nádobí – plný dřez se nedá používat. Při plné myčce odložit vedle na linku a pak do myčky, nebo hned umýt.</t>
+          <t>Když dochází jar, tablety do myčky, WC gel, toaletní papír nebo pytle do koše, tak to koupíš a hodíš do SettleUp.</t>
         </is>
       </c>
       <c r="D50" s="70" t="n"/>
       <c r="E50" s="70" t="n"/>
       <c r="F50" s="70" t="n"/>
     </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="67" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="B51" s="68" t="inlineStr">
-        <is>
-          <t>Spotřební materiál a chemie:</t>
-        </is>
-      </c>
-      <c r="C51" s="69" t="inlineStr">
-        <is>
-          <t>Když dochází jar, tablety do myčky, WC gel, toaletní papír nebo pytle do koše, tak to koupíš a hodíš do SettleUp.</t>
-        </is>
-      </c>
-      <c r="D51" s="70" t="n"/>
-      <c r="E51" s="70" t="n"/>
-      <c r="F51" s="70" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="37">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="C48:F48"/>
     <mergeCell ref="A46:F46"/>
-    <mergeCell ref="A18:F18"/>
     <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B18:F18"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="C49:F49"/>
+    <mergeCell ref="B11:F11"/>
     <mergeCell ref="B42:F42"/>
     <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B8:F8"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B29:F29"/>
+    <mergeCell ref="A10:F10"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B34:F34"/>
     <mergeCell ref="B28:F28"/>
@@ -6531,15 +6409,12 @@
     <mergeCell ref="A39:F39"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="C50:F50"/>
-    <mergeCell ref="A11:F11"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B15:F15"/>
     <mergeCell ref="B33:F33"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B36:F36"/>
-    <mergeCell ref="C51:F51"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="A25:F25"/>

</xml_diff>